<commit_message>
feat: show block name alongside branch in main inventory list
</commit_message>
<xml_diff>
--- a/sample-bulk-import-test-v2.xlsx
+++ b/sample-bulk-import-test-v2.xlsx
@@ -1,17 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{599E807B-AC65-48FA-B4CC-B28AFADC6884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Bulk Import Template" state="visible" r:id="rId4"/>
+    <sheet name="Bulk Import Template" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="38">
   <si>
     <t>Branch Name</t>
   </si>
@@ -110,19 +114,34 @@
   </si>
   <si>
     <t>Block C</t>
+  </si>
+  <si>
+    <t>Whiteboard2</t>
+  </si>
+  <si>
+    <t>Whiteboard3</t>
+  </si>
+  <si>
+    <t>Standard Desk2</t>
+  </si>
+  <si>
+    <t>First aid kit2</t>
+  </si>
+  <si>
+    <t>First aid kit3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -485,9 +504,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J10"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -498,7 +517,7 @@
     <col min="10" max="10" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -530,7 +549,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -558,11 +577,11 @@
       <c r="I2" t="s">
         <v>15</v>
       </c>
-      <c r="J2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J2">
+        <v>34645</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -570,7 +589,7 @@
         <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s">
         <v>13</v>
@@ -590,11 +609,11 @@
       <c r="I3" t="s">
         <v>15</v>
       </c>
-      <c r="J3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J3">
+        <v>45664</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -622,11 +641,11 @@
       <c r="I4" t="s">
         <v>22</v>
       </c>
-      <c r="J4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J4">
+        <v>6546</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -634,7 +653,7 @@
         <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="D5" t="s">
         <v>21</v>
@@ -654,11 +673,11 @@
       <c r="I5" t="s">
         <v>22</v>
       </c>
-      <c r="J5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J5">
+        <v>654645</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -666,7 +685,7 @@
         <v>24</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
         <v>21</v>
@@ -686,11 +705,11 @@
       <c r="I6" t="s">
         <v>22</v>
       </c>
-      <c r="J6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J6">
+        <v>654456</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -718,11 +737,11 @@
       <c r="I7" t="s">
         <v>26</v>
       </c>
-      <c r="J7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J7">
+        <v>654645</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>27</v>
       </c>
@@ -750,11 +769,11 @@
       <c r="I8" t="s">
         <v>31</v>
       </c>
-      <c r="J8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J8">
+        <v>654645</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>27</v>
       </c>
@@ -762,7 +781,7 @@
         <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="D9" t="s">
         <v>29</v>
@@ -782,11 +801,11 @@
       <c r="I9" t="s">
         <v>31</v>
       </c>
-      <c r="J9" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J9">
+        <v>654456</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -794,7 +813,7 @@
         <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="D10" t="s">
         <v>29</v>
@@ -814,12 +833,12 @@
       <c r="I10" t="s">
         <v>31</v>
       </c>
-      <c r="J10" t="s">
-        <v>16</v>
+      <c r="J10">
+        <v>654645</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>